<commit_message>
Update default PCE values to 1.0, 1.8, 2.5; format output report filename as YYYYMMDDHHMM; ensure UI dashboard loads latest generated report on custom PCE runs
</commit_message>
<xml_diff>
--- a/output/VD_traffic_report_20250522.xlsx
+++ b/output/VD_traffic_report_20250522.xlsx
@@ -471,12 +471,12 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -597,31 +597,31 @@
         <v>100</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>4044</v>
+        <v>6109</v>
       </c>
       <c r="G3" s="6" t="n">
-        <v>0.5465540540540541</v>
+        <v>0.8255405405405405</v>
       </c>
       <c r="H3" s="7" t="n">
-        <v>90.07775957098168</v>
+        <v>90.51340373679935</v>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="J3" s="4" t="n">
-        <v>6174</v>
+        <v>9847</v>
       </c>
       <c r="K3" s="6" t="n">
-        <v>0.8343918918918919</v>
+        <v>1.330675675675676</v>
       </c>
       <c r="L3" s="7" t="n">
-        <v>62.82014106583072</v>
+        <v>56.53251470079557</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>F4</t>
         </is>
       </c>
     </row>
@@ -648,31 +648,31 @@
         <v>100</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>5987</v>
+        <v>9628</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>0.8090202702702702</v>
+        <v>1.301081081081081</v>
       </c>
       <c r="H4" s="7" t="n">
-        <v>81.28432744446388</v>
+        <v>81.46104827146726</v>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="J4" s="4" t="n">
-        <v>3004</v>
+        <v>4884</v>
       </c>
       <c r="K4" s="6" t="n">
-        <v>0.4060135135135135</v>
+        <v>0.6600675675675676</v>
       </c>
       <c r="L4" s="7" t="n">
-        <v>87.36653805682217</v>
+        <v>86.91695721077654</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
@@ -699,31 +699,31 @@
         <v>100</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>3614</v>
+        <v>5712</v>
       </c>
       <c r="G5" s="6" t="n">
-        <v>0.4883108108108108</v>
+        <v>0.7718918918918919</v>
       </c>
       <c r="H5" s="7" t="n">
-        <v>91.10389221556886</v>
+        <v>91.13851167843563</v>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="J5" s="4" t="n">
-        <v>5284</v>
+        <v>8646</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>0.7140202702702703</v>
+        <v>1.168310810810811</v>
       </c>
       <c r="L5" s="7" t="n">
-        <v>49.12839554426422</v>
+        <v>43.59038699416858</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>F4</t>
         </is>
       </c>
     </row>
@@ -750,31 +750,31 @@
         <v>100</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>6104</v>
+        <v>9780</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>0.8248648648648649</v>
+        <v>1.321689189189189</v>
       </c>
       <c r="H6" s="7" t="n">
-        <v>90.49882720875684</v>
+        <v>90.39687795648061</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="J6" s="4" t="n">
-        <v>3058</v>
+        <v>4930</v>
       </c>
       <c r="K6" s="6" t="n">
-        <v>0.4132094594594595</v>
+        <v>0.6661486486486486</v>
       </c>
       <c r="L6" s="7" t="n">
-        <v>96.55135793871867</v>
+        <v>96.27051767676768</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>B1</t>
+          <t>C1</t>
         </is>
       </c>
     </row>
@@ -801,31 +801,31 @@
         <v>100</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>5093</v>
+        <v>7702</v>
       </c>
       <c r="G7" s="6" t="n">
-        <v>0.6882432432432433</v>
+        <v>1.040743243243243</v>
       </c>
       <c r="H7" s="7" t="n">
-        <v>88.13080304492334</v>
+        <v>87.20966105134971</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="J7" s="4" t="n">
-        <v>5838</v>
+        <v>8943</v>
       </c>
       <c r="K7" s="6" t="n">
-        <v>0.7888513513513513</v>
+        <v>1.208513513513513</v>
       </c>
       <c r="L7" s="7" t="n">
-        <v>52.30340299611615</v>
+        <v>42.36626676076217</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>F4</t>
         </is>
       </c>
     </row>
@@ -852,31 +852,31 @@
         <v>100</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>7069</v>
+        <v>11368</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>0.8365976331360947</v>
+        <v>1.345325443786982</v>
       </c>
       <c r="H8" s="7" t="n">
-        <v>54.84710561201944</v>
+        <v>55.51557233382769</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>F4</t>
         </is>
       </c>
       <c r="J8" s="4" t="n">
-        <v>4028</v>
+        <v>6660</v>
       </c>
       <c r="K8" s="6" t="n">
-        <v>0.4766568047337278</v>
+        <v>0.7881065088757396</v>
       </c>
       <c r="L8" s="7" t="n">
-        <v>74.6237292497748</v>
+        <v>81.95004604051566</v>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>C2</t>
         </is>
       </c>
     </row>
@@ -903,31 +903,31 @@
         <v>100</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>4954</v>
+        <v>7699</v>
       </c>
       <c r="G9" s="6" t="n">
-        <v>0.669527027027027</v>
+        <v>1.040405405405405</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>70.49615749026214</v>
+        <v>70.46290033817387</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="J9" s="4" t="n">
-        <v>5926</v>
+        <v>9268</v>
       </c>
       <c r="K9" s="6" t="n">
-        <v>0.8007432432432432</v>
+        <v>1.252364864864865</v>
       </c>
       <c r="L9" s="7" t="n">
-        <v>49.30457290767903</v>
+        <v>42.54301163362281</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>F4</t>
         </is>
       </c>
     </row>
@@ -954,31 +954,31 @@
         <v>100</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>8290</v>
+        <v>12650</v>
       </c>
       <c r="G10" s="6" t="n">
-        <v>0.9810059171597633</v>
+        <v>1.497041420118343</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>70.98018571324121</v>
+        <v>68.23834335337341</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="J10" s="4" t="n">
-        <v>4460</v>
+        <v>6962</v>
       </c>
       <c r="K10" s="6" t="n">
-        <v>0.5278698224852071</v>
+        <v>0.823905325443787</v>
       </c>
       <c r="L10" s="7" t="n">
-        <v>92.16088570331499</v>
+        <v>91.45247501742971</v>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>D1</t>
         </is>
       </c>
     </row>
@@ -1005,13 +1005,13 @@
         <v>100</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>9092</v>
+        <v>13583</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>1.344933431952663</v>
+        <v>2.009319526627219</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>76.88374796558939</v>
+        <v>76.7724537299875</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
@@ -1019,13 +1019,13 @@
         </is>
       </c>
       <c r="J11" s="4" t="n">
-        <v>9619</v>
+        <v>15738</v>
       </c>
       <c r="K11" s="6" t="n">
-        <v>1.42292899408284</v>
+        <v>2.328032544378698</v>
       </c>
       <c r="L11" s="7" t="n">
-        <v>55.27059394724066</v>
+        <v>55.87998056365403</v>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
@@ -1056,13 +1056,13 @@
         <v>100</v>
       </c>
       <c r="F12" s="4" t="n">
-        <v>13512</v>
+        <v>20956</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>2.370526315789474</v>
+        <v>3.67640350877193</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>66.57225031849593</v>
+        <v>62.04863955529549</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
@@ -1070,13 +1070,13 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>8211</v>
+        <v>13376</v>
       </c>
       <c r="K12" s="6" t="n">
-        <v>1.440570175438596</v>
+        <v>2.346578947368421</v>
       </c>
       <c r="L12" s="7" t="n">
-        <v>82.33293458414657</v>
+        <v>80.79281135531136</v>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
@@ -1107,13 +1107,13 @@
         <v>100</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>9092</v>
+        <v>13583</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>1.344933431952663</v>
+        <v>2.009319526627219</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>76.88374796558939</v>
+        <v>76.7724537299875</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
@@ -1121,13 +1121,13 @@
         </is>
       </c>
       <c r="J13" s="4" t="n">
-        <v>9619</v>
+        <v>15738</v>
       </c>
       <c r="K13" s="6" t="n">
-        <v>1.42292899408284</v>
+        <v>2.328032544378698</v>
       </c>
       <c r="L13" s="7" t="n">
-        <v>55.27059394724066</v>
+        <v>55.87998056365403</v>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
@@ -1158,13 +1158,13 @@
         <v>100</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>13512</v>
+        <v>20956</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>2.370526315789474</v>
+        <v>3.67640350877193</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>66.57225031849593</v>
+        <v>62.04863955529549</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
@@ -1172,13 +1172,13 @@
         </is>
       </c>
       <c r="J14" s="4" t="n">
-        <v>8211</v>
+        <v>13376</v>
       </c>
       <c r="K14" s="6" t="n">
-        <v>1.440570175438596</v>
+        <v>2.346578947368421</v>
       </c>
       <c r="L14" s="7" t="n">
-        <v>82.33293458414657</v>
+        <v>80.79281135531136</v>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
@@ -1209,31 +1209,31 @@
         <v>100</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>4566</v>
+        <v>6590</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>0.6754437869822485</v>
+        <v>0.9747781065088758</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>86.82795558458524</v>
+        <v>87.51951951951952</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>E2</t>
         </is>
       </c>
       <c r="J15" s="4" t="n">
-        <v>4231</v>
+        <v>6890</v>
       </c>
       <c r="K15" s="6" t="n">
-        <v>0.6258505917159763</v>
+        <v>1.019230769230769</v>
       </c>
       <c r="L15" s="7" t="n">
-        <v>85.03422882858312</v>
+        <v>83.19416547106647</v>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>F2</t>
         </is>
       </c>
     </row>
@@ -1260,31 +1260,31 @@
         <v>100</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>5961</v>
+        <v>8736</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>0.88176775147929</v>
+        <v>1.292233727810651</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>82.07081928188852</v>
+        <v>82.07114549915079</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="J16" s="4" t="n">
-        <v>3748</v>
+        <v>5620</v>
       </c>
       <c r="K16" s="6" t="n">
-        <v>0.5544748520710059</v>
+        <v>0.8313609467455622</v>
       </c>
       <c r="L16" s="7" t="n">
-        <v>69.23814655172414</v>
+        <v>68.478349317059</v>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>D3</t>
         </is>
       </c>
     </row>
@@ -1311,31 +1311,31 @@
         <v>100</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>4351</v>
+        <v>6642</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>0.6436020710059172</v>
+        <v>0.9824704142011834</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>98.46455938697318</v>
+        <v>99.22224775913583</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="J17" s="4" t="n">
-        <v>4052</v>
+        <v>6973</v>
       </c>
       <c r="K17" s="6" t="n">
-        <v>0.5994082840236686</v>
+        <v>1.031508875739645</v>
       </c>
       <c r="L17" s="7" t="n">
-        <v>95.58391036132444</v>
+        <v>94.55026109660574</v>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>F1</t>
         </is>
       </c>
     </row>
@@ -1362,10 +1362,10 @@
         <v>100</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>-810</v>
+        <v>0</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>-0.1198224852071006</v>
+        <v>0</v>
       </c>
       <c r="H18" s="7" t="n">
         <v>0</v>
@@ -1376,10 +1376,10 @@
         </is>
       </c>
       <c r="J18" s="4" t="n">
-        <v>-808</v>
+        <v>0</v>
       </c>
       <c r="K18" s="6" t="n">
-        <v>-0.1194896449704142</v>
+        <v>0</v>
       </c>
       <c r="L18" s="7" t="n">
         <v>0</v>
@@ -1413,31 +1413,31 @@
         <v>100</v>
       </c>
       <c r="F19" s="4" t="n">
-        <v>4959</v>
+        <v>7274</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>0.7336168639053254</v>
+        <v>1.075961538461538</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>87.40337299295368</v>
+        <v>88.82890070921985</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="J19" s="4" t="n">
-        <v>4212</v>
+        <v>7000</v>
       </c>
       <c r="K19" s="6" t="n">
-        <v>0.6230029585798816</v>
+        <v>1.035502958579882</v>
       </c>
       <c r="L19" s="7" t="n">
-        <v>50.85568930925767</v>
+        <v>68.99203000468823</v>
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>C4</t>
+          <t>F3</t>
         </is>
       </c>
     </row>
@@ -1464,31 +1464,31 @@
         <v>100</v>
       </c>
       <c r="F20" s="4" t="n">
-        <v>6526</v>
+        <v>9534</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>0.9653846153846154</v>
+        <v>1.41042899408284</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>77.27584891262877</v>
+        <v>75.95997836668469</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>E3</t>
+          <t>F3</t>
         </is>
       </c>
       <c r="J20" s="4" t="n">
-        <v>4031</v>
+        <v>6442</v>
       </c>
       <c r="K20" s="6" t="n">
-        <v>0.596301775147929</v>
+        <v>0.9529585798816568</v>
       </c>
       <c r="L20" s="7" t="n">
-        <v>92.26294474978305</v>
+        <v>91.59928168291431</v>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>E1</t>
         </is>
       </c>
     </row>
@@ -1515,13 +1515,13 @@
         <v>100</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>10737</v>
+        <v>15522</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>1.588313609467456</v>
+        <v>2.296153846153846</v>
       </c>
       <c r="H21" s="7" t="n">
-        <v>46.74627453185627</v>
+        <v>46.23509862778731</v>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
@@ -1529,17 +1529,17 @@
         </is>
       </c>
       <c r="J21" s="4" t="n">
-        <v>6038</v>
+        <v>9214</v>
       </c>
       <c r="K21" s="6" t="n">
-        <v>0.8931952662721894</v>
+        <v>1.362943786982248</v>
       </c>
       <c r="L21" s="7" t="n">
-        <v>27.92446393762183</v>
+        <v>35.01804032543332</v>
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>F5</t>
         </is>
       </c>
     </row>
@@ -1566,13 +1566,13 @@
         <v>100</v>
       </c>
       <c r="F22" s="4" t="n">
-        <v>16861</v>
+        <v>25092</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>2.49426775147929</v>
+        <v>3.711908284023669</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>79.68739726027397</v>
+        <v>78.1557994544746</v>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
@@ -1580,17 +1580,17 @@
         </is>
       </c>
       <c r="J22" s="4" t="n">
-        <v>12740</v>
+        <v>19153</v>
       </c>
       <c r="K22" s="6" t="n">
-        <v>1.884541420118343</v>
+        <v>2.833284023668639</v>
       </c>
       <c r="L22" s="7" t="n">
-        <v>79.82836784680472</v>
+        <v>80.11425206124852</v>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F2</t>
         </is>
       </c>
     </row>
@@ -1617,13 +1617,13 @@
         <v>100</v>
       </c>
       <c r="F23" s="4" t="n">
-        <v>10737</v>
+        <v>15522</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>1.588313609467456</v>
+        <v>2.296153846153846</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>46.74627453185627</v>
+        <v>46.23509862778731</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
@@ -1631,17 +1631,17 @@
         </is>
       </c>
       <c r="J23" s="4" t="n">
-        <v>6038</v>
+        <v>9214</v>
       </c>
       <c r="K23" s="6" t="n">
-        <v>0.8931952662721894</v>
+        <v>1.362943786982248</v>
       </c>
       <c r="L23" s="7" t="n">
-        <v>27.92446393762183</v>
+        <v>35.01804032543332</v>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>F5</t>
         </is>
       </c>
     </row>
@@ -1668,13 +1668,13 @@
         <v>100</v>
       </c>
       <c r="F24" s="4" t="n">
-        <v>16861</v>
+        <v>25092</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>2.49426775147929</v>
+        <v>3.711908284023669</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>79.68739726027397</v>
+        <v>78.1557994544746</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
@@ -1682,17 +1682,17 @@
         </is>
       </c>
       <c r="J24" s="4" t="n">
-        <v>12740</v>
+        <v>19153</v>
       </c>
       <c r="K24" s="6" t="n">
-        <v>1.884541420118343</v>
+        <v>2.833284023668639</v>
       </c>
       <c r="L24" s="7" t="n">
-        <v>79.82836784680472</v>
+        <v>80.11425206124852</v>
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>F2</t>
         </is>
       </c>
     </row>
@@ -1875,31 +1875,31 @@
         <v>50</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>2006</v>
+        <v>3505</v>
       </c>
       <c r="I3" s="6" t="n">
-        <v>0.5278947368421053</v>
+        <v>0.9223684210526316</v>
       </c>
       <c r="J3" s="7" t="n">
-        <v>72.53324742268042</v>
+        <v>72.54613030170529</v>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>E1</t>
         </is>
       </c>
       <c r="L3" s="4" t="n">
-        <v>3366</v>
+        <v>5993</v>
       </c>
       <c r="M3" s="6" t="n">
-        <v>0.8858552631578948</v>
+        <v>1.577105263157895</v>
       </c>
       <c r="N3" s="7" t="n">
-        <v>68.98093508851566</v>
+        <v>68.21115335868187</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>F1</t>
         </is>
       </c>
     </row>
@@ -1936,13 +1936,13 @@
         <v>50</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>3510</v>
+        <v>6070</v>
       </c>
       <c r="I4" s="6" t="n">
-        <v>1.169916666666667</v>
+        <v>2.0235</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>72.39959225280326</v>
+        <v>69.81695423855965</v>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
@@ -1950,17 +1950,17 @@
         </is>
       </c>
       <c r="L4" s="4" t="n">
-        <v>1805</v>
+        <v>2921</v>
       </c>
       <c r="M4" s="6" t="n">
-        <v>0.6015833333333334</v>
+        <v>0.9736666666666667</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>75.19532363843742</v>
+        <v>75.67765567765568</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>E1</t>
         </is>
       </c>
     </row>

</xml_diff>